<commit_message>
Testando recursos da biblioteca openpyxl
</commit_message>
<xml_diff>
--- a/Python_Automacao/Lendo Excel.xlsx
+++ b/Python_Automacao/Lendo Excel.xlsx
@@ -2,16 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
   <sheets>
     <sheet name="Nomes" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Dias da semana" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Doces" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -136,44 +133,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Yu Gothic Light"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -203,12 +200,12 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Yu Gothic"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -247,142 +244,201 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
+                <a:tint val="100000"/>
                 <a:shade val="100000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
@@ -392,8 +448,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
+  <cols>
+    <col width="17.57142857142857" customWidth="1" min="1" max="1"/>
+    <col width="13.57142857142857" customWidth="1" min="2" max="24"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -457,8 +517,49 @@
         <v>12</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Taíta</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Lincon</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Rozane</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Paulo César</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
@@ -469,10 +570,11 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
-    <col width="13.44140625" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="13.88671875" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="13.42857142857143" customWidth="1" min="1" max="1"/>
+    <col width="13.85714285714286" customWidth="1" min="2" max="2"/>
+    <col width="13.57142857142857" customWidth="1" min="3" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -558,7 +660,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.787401575" bottom="0.787401575" header="0.31496062" footer="0.31496062"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
@@ -569,9 +672,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
-    <col width="17.44140625" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="21.71428571428572" customWidth="1" min="1" max="1"/>
+    <col width="13.57142857142857" customWidth="1" min="2" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -617,6 +721,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.787401575" bottom="0.787401575" header="0.31496062" footer="0.31496062"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>